<commit_message>
Making changes in the  featuregenerator.java file
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/loginData.xlsx
+++ b/src/test/resources/testdata/loginData.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA696225-F703-41AB-A955-52FA4562C183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>usename</t>
   </si>
@@ -31,9 +32,7 @@
     <t>Password123!</t>
   </si>
   <si>
-    <r>
-      <t>success</t>
-    </r>
+    <t>fail</t>
   </si>
   <si>
     <t>wronguser</t>
@@ -49,65 +48,27 @@
   </si>
   <si>
     <t>nagpur</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF000000"/>
-      </rPr>
-      <t>testuser</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF000000"/>
-      </rPr>
-      <t>Password123!</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>fail</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF000000"/>
-      </rPr>
-      <t>success</t>
-    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -436,9 +397,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.55" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="2" width="32" customWidth="1"/>
   </cols>
@@ -487,75 +448,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>